<commit_message>
fix: sync Vercel frontend build with Render live backend URL and updated header components
</commit_message>
<xml_diff>
--- a/tests/reports/Blogify_E2E_Test_Report.xlsx
+++ b/tests/reports/Blogify_E2E_Test_Report.xlsx
@@ -39,7 +39,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -54,11 +54,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0016A34A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DC2626"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -93,9 +88,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -481,7 +473,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-22 15:13:25</t>
+          <t>2026-07-31 17:25:17</t>
         </is>
       </c>
     </row>
@@ -492,7 +484,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -502,7 +494,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -512,7 +504,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -533,7 +525,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>85.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -551,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -605,7 +597,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_011_register_page_loads</t>
+          <t>selenium_tests/test_01_homepage.py::TestHomepage::test_tc_s_001_homepage_loads_successfully</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -614,7 +606,7 @@
         </is>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0.31</v>
+        <v>0.169</v>
       </c>
       <c r="F2" s="4" t="inlineStr"/>
     </row>
@@ -629,7 +621,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_012_register_all_fields_present</t>
+          <t>selenium_tests/test_01_homepage.py::TestHomepage::test_tc_s_002_hero_section_visible</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -638,7 +630,7 @@
         </is>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.347</v>
+        <v>0.532</v>
       </c>
       <c r="F3" s="4" t="inlineStr"/>
     </row>
@@ -653,7 +645,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_013_register_empty_submit_shows_error</t>
+          <t>selenium_tests/test_01_homepage.py::TestHomepage::test_tc_s_003_navbar_visible</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -662,7 +654,7 @@
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1.378</v>
+        <v>0.476</v>
       </c>
       <c r="F4" s="4" t="inlineStr"/>
     </row>
@@ -677,7 +669,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_014_register_weak_password_error</t>
+          <t>selenium_tests/test_01_homepage.py::TestHomepage::test_tc_s_004_explore_link_in_navbar</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -686,7 +678,7 @@
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.543</v>
+        <v>0.255</v>
       </c>
       <c r="F5" s="4" t="inlineStr"/>
     </row>
@@ -701,7 +693,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_015_register_strong_password_shown</t>
+          <t>selenium_tests/test_01_homepage.py::TestHomepage::test_tc_s_005_login_button_in_navbar</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -710,7 +702,7 @@
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.595</v>
+        <v>0.477</v>
       </c>
       <c r="F6" s="4" t="inlineStr"/>
     </row>
@@ -725,7 +717,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_016_register_password_mismatch_error</t>
+          <t>selenium_tests/test_01_homepage.py::TestHomepage::test_tc_s_006_homepage_has_blog_section</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -734,7 +726,7 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>1.732</v>
+        <v>0.136</v>
       </c>
       <c r="F7" s="4" t="inlineStr"/>
     </row>
@@ -749,7 +741,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_017_register_success_redirects_to_login</t>
+          <t>selenium_tests/test_01_homepage.py::TestHomepage::test_tc_s_007_footer_is_displayed</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -758,7 +750,7 @@
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>4.581</v>
+        <v>1.178</v>
       </c>
       <c r="F8" s="4" t="inlineStr"/>
     </row>
@@ -773,7 +765,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_018_register_duplicate_email_error</t>
+          <t>selenium_tests/test_01_homepage.py::TestHomepage::test_tc_s_008_page_title_is_correct</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -782,7 +774,7 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>4.382</v>
+        <v>0.162</v>
       </c>
       <c r="F9" s="4" t="inlineStr"/>
     </row>
@@ -797,7 +789,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_019_login_page_loads</t>
+          <t>selenium_tests/test_01_homepage.py::TestHomepage::test_tc_s_009_meta_description_exists</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -806,7 +798,7 @@
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0.367</v>
+        <v>0.457</v>
       </c>
       <c r="F10" s="4" t="inlineStr"/>
     </row>
@@ -821,7 +813,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_020_login_empty_form_blocked</t>
+          <t>selenium_tests/test_01_homepage.py::TestHomepage::test_tc_s_010_get_started_button_visible</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -830,267 +822,9 @@
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>1.452</v>
+        <v>0.513</v>
       </c>
       <c r="F11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>TEST_TC_S</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_021_login_wrong_credentials_error</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>3.765</v>
-      </c>
-      <c r="F12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>TEST_TC_S</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_022_valid_login_redirects</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>33.291</v>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>E   selenium.common.exceptions.TimeoutException: Message:</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>TEST_TC_S</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_023_admin_blocked_on_public_login</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>3.898</v>
-      </c>
-      <c r="F14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>TEST_TC_S</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_024_forgot_password_link_navigates</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>0.468</v>
-      </c>
-      <c r="F15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>TEST_TC_S</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_025_forgot_password_sends_email</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>4.871</v>
-      </c>
-      <c r="F16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>TEST_TC_S</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_026_login_shows_password_toggle</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>1.373</v>
-      </c>
-      <c r="F17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>TEST_TC_S</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_027_register_link_on_login_page</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>0.504</v>
-      </c>
-      <c r="F18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>TEST_TC_S</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_028_session_token_stored_in_localstorage</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>32.395</v>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>E   selenium.common.exceptions.TimeoutException: Message:</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>TEST_TC_S</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_029_logout_clears_localstorage</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>21.757</v>
-      </c>
-      <c r="F20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>TEST_TC_S</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>selenium_tests/test_02_auth.py::TestAuth::test_tc_s_030_registered_user_login_flow</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>11.734</v>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>E   AssertionError: E2E register-&gt;login flow failed
-    assert ('/login' not in 'http://loca...t:5173/login'
-      '/login' is contained here:
-        http://localhost:5173/login
-      ?                      ++++++ or None is not None)
-     +  where None = execute_script("return window.localStorage.getItem('token');")
-     +    where execute_script = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="daf9883dbe273fa8f45355dbff921c53")&gt;.execute_script</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>